<commit_message>
The --my-station was promoting fields not intended to be promoted.  Removed it and will use the keywords direcly.  For the Excel version, a separate worksheet, MISC, will support the same updates as the cSV.  The other worksheet names are kept for the use case of someone cutting and pasting from QRZ into Excel.
</commit_message>
<xml_diff>
--- a/qrz_errors_example.xlsx
+++ b/qrz_errors_example.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\radio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D8F1BC-3DC5-449F-8ED1-6BAA0B3F8ACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{075D0FDD-DABD-41C3-9E10-CFFA9BEEA215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12252" yWindow="2496" windowWidth="20448" windowHeight="18636" activeTab="2" xr2:uid="{42681BCE-169B-4755-B878-5A88229D2996}"/>
+    <workbookView xWindow="5271" yWindow="1954" windowWidth="18515" windowHeight="11555" activeTab="3" xr2:uid="{42681BCE-169B-4755-B878-5A88229D2996}"/>
   </bookViews>
   <sheets>
     <sheet name="Grids" sheetId="1" r:id="rId1"/>
     <sheet name="State" sheetId="2" r:id="rId2"/>
     <sheet name="County" sheetId="3" r:id="rId3"/>
+    <sheet name="MISC" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="47">
   <si>
     <t>QSO Date</t>
   </si>
@@ -137,6 +138,48 @@
   </si>
   <si>
     <t>Pima County, AZ</t>
+  </si>
+  <si>
+    <t>field</t>
+  </si>
+  <si>
+    <t>qso_date</t>
+  </si>
+  <si>
+    <t>qso_with</t>
+  </si>
+  <si>
+    <t>new_value</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>GRIDSQUARE</t>
+  </si>
+  <si>
+    <t>W1TF</t>
+  </si>
+  <si>
+    <t>FN42</t>
+  </si>
+  <si>
+    <t>WG0Y</t>
+  </si>
+  <si>
+    <t>DM35</t>
+  </si>
+  <si>
+    <t>MY_GRIDSQUARE</t>
+  </si>
+  <si>
+    <t>CN97an</t>
+  </si>
+  <si>
+    <t>STATE</t>
+  </si>
+  <si>
+    <t>AZ</t>
   </si>
 </sst>
 </file>
@@ -180,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -194,6 +237,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -529,15 +573,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADAEC160-A63B-4F0F-9FF4-ED39A651243C}">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.15"/>
   <cols>
-    <col min="1" max="1" width="15.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.2109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.78515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.3984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.19921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.2109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -606,14 +650,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE3882D1-59B4-4F0C-A382-96693C27E013}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.15"/>
   <cols>
-    <col min="1" max="1" width="15.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.2109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.78515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -684,9 +728,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3906EBB6-D3D7-4B9B-9A24-22333A4E538E}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.15"/>
   <cols>
-    <col min="1" max="1" width="15.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.2109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="28.5" bestFit="1" customWidth="1"/>
   </cols>
@@ -819,4 +863,107 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6D554C5-06A4-457E-A07E-37539418E6CF}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="14.15"/>
+  <cols>
+    <col min="1" max="1" width="16.92578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.0703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="5">
+        <v>46085.84375</v>
+      </c>
+      <c r="C2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="5">
+        <v>46127.977083333331</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="5">
+        <v>46085.84375</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="5">
+        <v>46127.977083333331</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="5">
+        <v>46127.977083333331</v>
+      </c>
+      <c r="C6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>